<commit_message>
#23 R129 removed. PDF and BOM updated
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_MCM_v1.61/Deliverables/BOM/Client-BOM-OFP_MCM_v1.61.xlsx
+++ b/Design-Files/OFP_MCM_v1.61/Deliverables/BOM/Client-BOM-OFP_MCM_v1.61.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\nabilfesal-smartmeter-hw\Design-Files\OFP_MCM_v1.61\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D1EFDA-6CDD-4679-9A0E-5EB4DBFED774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC3AAC01-2AA3-4777-BDF2-CC25C257692D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1935,12 +1935,6 @@
     <t>Part number updated. Switch height increased by 1mm.</t>
   </si>
   <si>
-    <t>R49, R59, R62, R73, R123, R124, R125, R126, R127, R129</t>
-  </si>
-  <si>
-    <t>R123, R124, R125, R126, R127, R129 added.</t>
-  </si>
-  <si>
     <t>YSPI0518S-4R7M</t>
   </si>
   <si>
@@ -2005,6 +1999,12 @@
   </si>
   <si>
     <t>47uF 25V 150mΩ@100kHz ±10% CASE-D-7343-31(mm) Tantalum Capacitors ROHS</t>
+  </si>
+  <si>
+    <t>R49, R59, R62, R73, R123, R124, R125, R126, R127</t>
+  </si>
+  <si>
+    <t>R123, R124, R125, R126, R127 added.</t>
   </si>
 </sst>
 </file>
@@ -3672,16 +3672,16 @@
         <v>21</v>
       </c>
       <c r="D36" s="12" t="s">
+        <v>651</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>654</v>
+      </c>
+      <c r="F36" s="12" t="s">
         <v>653</v>
       </c>
-      <c r="E36" s="13" t="s">
-        <v>656</v>
-      </c>
-      <c r="F36" s="12" t="s">
-        <v>655</v>
-      </c>
       <c r="G36" s="13" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="H36" s="12" t="s">
         <v>148</v>
@@ -4269,13 +4269,13 @@
         <v>231</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>240</v>
@@ -4287,7 +4287,7 @@
         <v>3</v>
       </c>
       <c r="K54" s="9" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -4719,19 +4719,19 @@
         <v>278</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>281</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="I68" s="10" t="s">
         <v>155</v>
@@ -5105,7 +5105,7 @@
         <v>293</v>
       </c>
       <c r="D80" s="12" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="E80" s="13" t="s">
         <v>340</v>
@@ -5126,7 +5126,7 @@
         <v>7</v>
       </c>
       <c r="K80" s="12" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -5299,7 +5299,7 @@
         <v>293</v>
       </c>
       <c r="D86" s="12" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="E86" s="13" t="s">
         <v>363</v>
@@ -5459,7 +5459,7 @@
         <v>293</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>363</v>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="K93" s="9"/>
     </row>
-    <row r="94" spans="1:11" ht="24">
+    <row r="94" spans="1:11">
       <c r="A94" s="2"/>
       <c r="B94" s="7">
         <f t="shared" si="2"/>
@@ -5557,7 +5557,7 @@
         <v>293</v>
       </c>
       <c r="D94" s="12" t="s">
-        <v>633</v>
+        <v>655</v>
       </c>
       <c r="E94" s="13" t="s">
         <v>388</v>
@@ -5575,10 +5575,10 @@
         <v>390</v>
       </c>
       <c r="J94" s="12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K94" s="12" t="s">
-        <v>634</v>
+        <v>656</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -5907,7 +5907,7 @@
         <v>293</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>429</v>
@@ -5928,7 +5928,7 @@
         <v>7</v>
       </c>
       <c r="K105" s="9" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -5941,7 +5941,7 @@
         <v>293</v>
       </c>
       <c r="D106" s="12" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="E106" s="13" t="s">
         <v>432</v>
@@ -5962,7 +5962,7 @@
         <v>3</v>
       </c>
       <c r="K106" s="12" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -7333,10 +7333,10 @@
       <c r="A149" s="2"/>
       <c r="B149" s="7"/>
       <c r="C149" s="8" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D149" s="9" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E149" s="10" t="s">
         <v>155</v>
@@ -7351,7 +7351,7 @@
         <v>155</v>
       </c>
       <c r="I149" s="10" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="J149" s="9">
         <v>1</v>

</xml_diff>